<commit_message>
Update sales.xlsx from DailyStock
</commit_message>
<xml_diff>
--- a/data/sales.xlsx
+++ b/data/sales.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2572" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2586" uniqueCount="132">
   <si>
     <t>ITEM NAME</t>
   </si>
@@ -290,6 +290,12 @@
     <t>2026-08-31</t>
   </si>
   <si>
+    <t>2026-09-01</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
     <t>2026-08-30</t>
   </si>
   <si>
@@ -324,9 +330,6 @@
   </si>
   <si>
     <t>CLOSING VALUE</t>
-  </si>
-  <si>
-    <t>2026-09</t>
   </si>
   <si>
     <t>SALES - 1 AUGUST 2026</t>
@@ -408,6 +411,9 @@
   </si>
   <si>
     <t>SALES - 31 AUGUST 2026</t>
+  </si>
+  <si>
+    <t>SALES - 1 SEPTEMBER 2026</t>
   </si>
 </sst>
 </file>
@@ -1473,7 +1479,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F396"/>
+  <dimension ref="A1:F397"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -9344,6 +9350,26 @@
       </c>
       <c r="F396">
         <v>150</v>
+      </c>
+    </row>
+    <row r="397" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A397" t="s">
+        <v>90</v>
+      </c>
+      <c r="B397" t="s">
+        <v>91</v>
+      </c>
+      <c r="C397" t="s">
+        <v>5</v>
+      </c>
+      <c r="D397">
+        <v>180</v>
+      </c>
+      <c r="E397">
+        <v>4</v>
+      </c>
+      <c r="F397">
+        <v>720</v>
       </c>
     </row>
   </sheetData>
@@ -9574,7 +9600,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B16" t="s">
         <v>64</v>
@@ -9586,15 +9612,15 @@
         <v>-200</v>
       </c>
       <c r="E16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F16" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B17" t="s">
         <v>64</v>
@@ -9606,10 +9632,10 @@
         <v>-50</v>
       </c>
       <c r="E17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -9682,10 +9708,10 @@
         <v>-900</v>
       </c>
       <c r="E22" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F22" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -9752,7 +9778,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E540"/>
+  <dimension ref="A1:E547"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -9764,7 +9790,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -9973,13 +9999,13 @@
     </row>
     <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D15" s="4">
         <v>41</v>
@@ -9990,7 +10016,7 @@
     </row>
     <row r="18" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -10301,13 +10327,13 @@
     </row>
     <row r="38" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B38" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D38" s="4">
         <v>117</v>
@@ -10318,7 +10344,7 @@
     </row>
     <row r="41" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -10595,13 +10621,13 @@
     </row>
     <row r="59" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B59" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C59" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D59" s="4">
         <v>246</v>
@@ -10612,7 +10638,7 @@
     </row>
     <row r="62" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -10906,13 +10932,13 @@
     </row>
     <row r="81" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B81" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C81" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C81" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D81" s="4">
         <v>36</v>
@@ -10923,7 +10949,7 @@
     </row>
     <row r="84" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="86" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11149,13 +11175,13 @@
     </row>
     <row r="99" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B99" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C99" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D99" s="4">
         <v>68</v>
@@ -11166,7 +11192,7 @@
     </row>
     <row r="102" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="104" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11426,13 +11452,13 @@
     </row>
     <row r="119" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B119" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C119" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C119" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D119" s="4">
         <v>92</v>
@@ -11443,7 +11469,7 @@
     </row>
     <row r="122" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="124" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11788,13 +11814,13 @@
     </row>
     <row r="144" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B144" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C144" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C144" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D144" s="4">
         <v>73</v>
@@ -11805,7 +11831,7 @@
     </row>
     <row r="147" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="149" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12082,13 +12108,13 @@
     </row>
     <row r="165" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B165" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C165" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C165" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D165" s="4">
         <v>150</v>
@@ -12099,7 +12125,7 @@
     </row>
     <row r="168" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="170" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12427,13 +12453,13 @@
     </row>
     <row r="189" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B189" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C189" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C189" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D189" s="4">
         <v>52</v>
@@ -12444,7 +12470,7 @@
     </row>
     <row r="192" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="194" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12704,13 +12730,13 @@
     </row>
     <row r="209" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B209" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C209" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C209" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D209" s="4">
         <v>51</v>
@@ -12721,7 +12747,7 @@
     </row>
     <row r="212" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="214" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -13049,13 +13075,13 @@
     </row>
     <row r="233" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A233" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B233" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C233" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C233" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D233" s="4">
         <v>109</v>
@@ -13066,7 +13092,7 @@
     </row>
     <row r="236" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A236" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="238" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -13326,13 +13352,13 @@
     </row>
     <row r="253" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A253" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B253" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C253" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C253" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D253" s="4">
         <v>55</v>
@@ -13343,7 +13369,7 @@
     </row>
     <row r="256" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A256" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="258" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -13586,13 +13612,13 @@
     </row>
     <row r="272" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A272" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B272" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C272" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C272" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D272" s="4">
         <v>38</v>
@@ -13603,7 +13629,7 @@
     </row>
     <row r="275" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A275" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="277" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -13914,13 +13940,13 @@
     </row>
     <row r="295" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A295" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B295" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C295" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C295" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D295" s="4">
         <v>98</v>
@@ -13931,7 +13957,7 @@
     </row>
     <row r="298" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A298" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="300" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -14259,13 +14285,13 @@
     </row>
     <row r="319" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A319" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B319" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C319" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C319" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D319" s="4">
         <v>49</v>
@@ -14276,7 +14302,7 @@
     </row>
     <row r="322" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A322" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="324" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -14587,13 +14613,13 @@
     </row>
     <row r="342" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A342" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B342" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C342" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C342" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D342" s="4">
         <v>113</v>
@@ -14604,7 +14630,7 @@
     </row>
     <row r="345" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A345" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="347" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -14932,13 +14958,13 @@
     </row>
     <row r="366" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A366" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B366" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C366" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C366" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D366" s="4">
         <v>84</v>
@@ -14949,7 +14975,7 @@
     </row>
     <row r="369" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A369" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="371" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -15260,13 +15286,13 @@
     </row>
     <row r="389" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A389" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B389" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C389" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C389" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D389" s="4">
         <v>86</v>
@@ -15277,7 +15303,7 @@
     </row>
     <row r="392" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A392" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="394" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -15520,13 +15546,13 @@
     </row>
     <row r="408" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A408" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B408" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C408" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C408" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D408" s="4">
         <v>39</v>
@@ -15537,7 +15563,7 @@
     </row>
     <row r="411" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A411" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="413" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -15831,13 +15857,13 @@
     </row>
     <row r="430" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A430" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B430" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C430" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C430" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D430" s="4">
         <v>82</v>
@@ -15848,7 +15874,7 @@
     </row>
     <row r="433" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A433" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="435" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -16125,13 +16151,13 @@
     </row>
     <row r="451" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A451" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B451" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C451" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C451" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D451" s="4">
         <v>95</v>
@@ -16142,7 +16168,7 @@
     </row>
     <row r="454" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A454" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="456" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -16436,13 +16462,13 @@
     </row>
     <row r="473" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A473" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B473" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C473" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C473" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D473" s="4">
         <v>63</v>
@@ -16453,7 +16479,7 @@
     </row>
     <row r="476" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A476" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="478" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -16713,13 +16739,13 @@
     </row>
     <row r="493" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A493" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B493" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C493" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C493" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D493" s="4">
         <v>35</v>
@@ -16730,7 +16756,7 @@
     </row>
     <row r="496" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A496" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="498" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -17041,13 +17067,13 @@
     </row>
     <row r="516" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A516" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B516" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C516" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C516" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D516" s="4">
         <v>96</v>
@@ -17058,7 +17084,7 @@
     </row>
     <row r="519" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A519" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="521" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -17386,19 +17412,75 @@
     </row>
     <row r="540" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A540" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B540" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C540" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="C540" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="D540" s="4">
         <v>147</v>
       </c>
       <c r="E540" s="4">
         <v>4147</v>
+      </c>
+    </row>
+    <row r="543" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A543" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="545" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A545" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B545" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C545" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D545" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E545" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="546" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A546" t="s">
+        <v>90</v>
+      </c>
+      <c r="B546" t="s">
+        <v>5</v>
+      </c>
+      <c r="C546">
+        <v>180</v>
+      </c>
+      <c r="D546">
+        <v>4</v>
+      </c>
+      <c r="E546">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="547" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A547" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B547" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C547" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D547" s="4">
+        <v>4</v>
+      </c>
+      <c r="E547" s="4">
+        <v>720</v>
       </c>
     </row>
   </sheetData>
@@ -17439,31 +17521,31 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>62</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -19764,7 +19846,7 @@
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B58" t="s">
         <v>3</v>
@@ -19805,7 +19887,7 @@
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B59" t="s">
         <v>4</v>
@@ -19846,7 +19928,7 @@
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B60" t="s">
         <v>5</v>
@@ -19873,21 +19955,21 @@
         <v>6120</v>
       </c>
       <c r="J60">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K60">
-        <v>0</v>
+        <v>720</v>
       </c>
       <c r="L60">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="M60">
-        <v>6120</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B61" t="s">
         <v>6</v>
@@ -19928,7 +20010,7 @@
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B62" t="s">
         <v>7</v>
@@ -19969,7 +20051,7 @@
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B63" t="s">
         <v>8</v>
@@ -20010,7 +20092,7 @@
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B64" t="s">
         <v>9</v>
@@ -20051,7 +20133,7 @@
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B65" t="s">
         <v>10</v>
@@ -20092,7 +20174,7 @@
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B66" t="s">
         <v>11</v>
@@ -20133,7 +20215,7 @@
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B67" t="s">
         <v>12</v>
@@ -20174,7 +20256,7 @@
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B68" t="s">
         <v>13</v>
@@ -20215,7 +20297,7 @@
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B69" t="s">
         <v>14</v>
@@ -20256,7 +20338,7 @@
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B70" t="s">
         <v>15</v>
@@ -20297,7 +20379,7 @@
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B71" t="s">
         <v>16</v>
@@ -20338,7 +20420,7 @@
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B72" t="s">
         <v>17</v>
@@ -20379,7 +20461,7 @@
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B73" t="s">
         <v>18</v>
@@ -20420,7 +20502,7 @@
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B74" t="s">
         <v>19</v>
@@ -20461,7 +20543,7 @@
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B75" t="s">
         <v>20</v>
@@ -20502,7 +20584,7 @@
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B76" t="s">
         <v>21</v>
@@ -20543,7 +20625,7 @@
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B77" t="s">
         <v>22</v>
@@ -20584,7 +20666,7 @@
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B78" t="s">
         <v>23</v>
@@ -20625,7 +20707,7 @@
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B79" t="s">
         <v>24</v>
@@ -20666,7 +20748,7 @@
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B80" t="s">
         <v>25</v>
@@ -20707,7 +20789,7 @@
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B81" t="s">
         <v>26</v>
@@ -20748,7 +20830,7 @@
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B82" t="s">
         <v>27</v>
@@ -20789,7 +20871,7 @@
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B83" t="s">
         <v>28</v>
@@ -20830,7 +20912,7 @@
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B84" t="s">
         <v>29</v>
@@ -20871,7 +20953,7 @@
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B85" t="s">
         <v>30</v>
@@ -20912,7 +20994,7 @@
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B86" t="s">
         <v>31</v>
@@ -20953,7 +21035,7 @@
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B87" t="s">
         <v>32</v>
@@ -20994,7 +21076,7 @@
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B88" t="s">
         <v>33</v>
@@ -21035,7 +21117,7 @@
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B89" t="s">
         <v>34</v>
@@ -21076,7 +21158,7 @@
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B90" t="s">
         <v>35</v>
@@ -21117,7 +21199,7 @@
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B91" t="s">
         <v>66</v>
@@ -21158,7 +21240,7 @@
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B92" t="s">
         <v>37</v>
@@ -21199,7 +21281,7 @@
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B93" t="s">
         <v>38</v>
@@ -21240,7 +21322,7 @@
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B94" t="s">
         <v>39</v>
@@ -21281,7 +21363,7 @@
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B95" t="s">
         <v>40</v>
@@ -21322,7 +21404,7 @@
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B96" t="s">
         <v>41</v>
@@ -21363,7 +21445,7 @@
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B97" t="s">
         <v>42</v>
@@ -21404,7 +21486,7 @@
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B98" t="s">
         <v>43</v>
@@ -21445,7 +21527,7 @@
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B99" t="s">
         <v>44</v>
@@ -21486,7 +21568,7 @@
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B100" t="s">
         <v>45</v>
@@ -21527,7 +21609,7 @@
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B101" t="s">
         <v>46</v>
@@ -21568,7 +21650,7 @@
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B102" t="s">
         <v>47</v>
@@ -21609,7 +21691,7 @@
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B103" t="s">
         <v>48</v>
@@ -21650,7 +21732,7 @@
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B104" t="s">
         <v>49</v>
@@ -21691,7 +21773,7 @@
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B105" t="s">
         <v>50</v>
@@ -21732,7 +21814,7 @@
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B106" t="s">
         <v>51</v>
@@ -21773,7 +21855,7 @@
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B107" t="s">
         <v>52</v>
@@ -21814,7 +21896,7 @@
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B108" t="s">
         <v>53</v>
@@ -21855,7 +21937,7 @@
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B109" t="s">
         <v>54</v>
@@ -21896,7 +21978,7 @@
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B110" t="s">
         <v>55</v>
@@ -21937,7 +22019,7 @@
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B111" t="s">
         <v>56</v>
@@ -21978,7 +22060,7 @@
     </row>
     <row r="112" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B112" t="s">
         <v>57</v>
@@ -22019,7 +22101,7 @@
     </row>
     <row r="113" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B113" t="s">
         <v>58</v>

</xml_diff>